<commit_message>
Select six common skill sprites or custom assets and configure tint from Excel
</commit_message>
<xml_diff>
--- a/Docs/SkillTemplates/スキル定義テンプレート.xlsx
+++ b/Docs/SkillTemplates/スキル定義テンプレート.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="スキル" sheetId="1" r:id="Rc2ad8614dddb470c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="モンスター列追加例" sheetId="2" r:id="R89d311b040f546f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入力ガイド" sheetId="3" r:id="R0051bf4f84624bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="スキル" sheetId="1" r:id="R0bfbeb24d8554b70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="モンスター列追加例" sheetId="2" r:id="R854b05576e3b4dc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="入力ガイド" sheetId="3" r:id="Rac2abcb45beb43fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="0.0##"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -90,8 +90,18 @@
       <x:sz val="11"/>
       <x:name val="Noto Sans JP"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF203864"/>
+      <x:name val="Noto Sans JP"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF172033"/>
+      <x:name val="Noto Sans JP"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="40">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -203,6 +213,91 @@
         <x:fgColor rgb="FFFFF3D5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF3D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF703F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF76FFB0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFE6A6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFBE55"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF8EEDCF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE3A15C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFB492FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF9DFF57"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF5030"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF72DBFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC18AFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBD70FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF6B38"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF70FFAC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF83BCFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF203864"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -216,7 +311,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="108">
+  <x:cellXfs count="143">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -459,6 +554,91 @@
     <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="11" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="12" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -921,10 +1101,11 @@
     <x:col min="121" max="121" width="22" hidden="0" customWidth="1"/>
     <x:col min="122" max="122" width="22" hidden="0" customWidth="1"/>
     <x:col min="123" max="123" width="22" hidden="0" customWidth="1"/>
-    <x:col min="124" max="124" width="22" hidden="0" customWidth="1"/>
+    <x:col min="124" max="124" width="24" hidden="0" customWidth="1"/>
     <x:col min="125" max="125" width="26" hidden="0" customWidth="1"/>
     <x:col min="126" max="126" width="26" hidden="0" customWidth="1"/>
     <x:col min="127" max="127" width="26" hidden="0" customWidth="1"/>
+    <x:col min="128" max="128" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="55" customHeight="1">
@@ -1297,17 +1478,20 @@
       <x:c r="DS1" s="87" t="str">
         <x:v>パッシブ3_効果量</x:v>
       </x:c>
-      <x:c r="DT1" s="98" t="str">
-        <x:v>発射物_画像番号</x:v>
-      </x:c>
-      <x:c r="DU1" s="104" t="str">
+      <x:c r="DT1" s="87" t="str">
+        <x:v>発射物_素材</x:v>
+      </x:c>
+      <x:c r="DU1" s="87" t="str">
         <x:v>発射物_範囲に表示を合わせる</x:v>
       </x:c>
-      <x:c r="DV1" s="104" t="str">
+      <x:c r="DV1" s="87" t="str">
         <x:v>発射物_爆発拡大秒</x:v>
       </x:c>
-      <x:c r="DW1" s="104" t="str">
+      <x:c r="DW1" s="87" t="str">
         <x:v>発射物_爆発開始倍率</x:v>
+      </x:c>
+      <x:c r="DX1" s="87" t="str">
+        <x:v>発射物_固有スプライト</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
@@ -1635,8 +1819,8 @@
       <x:c r="DE2" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF2" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF2" s="111" t="str">
+        <x:v>#FF703FFF</x:v>
       </x:c>
       <x:c r="DG2" s="45" t="n">
         <x:v>60</x:v>
@@ -1665,8 +1849,8 @@
       <x:c r="DQ2" s="88"/>
       <x:c r="DR2" s="88"/>
       <x:c r="DS2" s="88"/>
-      <x:c r="DT2" s="100" t="n">
-        <x:v>1</x:v>
+      <x:c r="DT2" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU2" s="106" t="str">
         <x:v>有効</x:v>
@@ -1677,6 +1861,7 @@
       <x:c r="DW2" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX2" s="109"/>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="9" t="str">
@@ -2003,8 +2188,8 @@
       <x:c r="DE3" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF3" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF3" s="113" t="str">
+        <x:v>#76FFB0FF</x:v>
       </x:c>
       <x:c r="DG3" s="45" t="n">
         <x:v>60</x:v>
@@ -2033,8 +2218,8 @@
       <x:c r="DQ3" s="88"/>
       <x:c r="DR3" s="88"/>
       <x:c r="DS3" s="88"/>
-      <x:c r="DT3" s="100" t="n">
-        <x:v>2</x:v>
+      <x:c r="DT3" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU3" s="106" t="str">
         <x:v>有効</x:v>
@@ -2045,6 +2230,7 @@
       <x:c r="DW3" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX3" s="109"/>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="9" t="str">
@@ -2371,8 +2557,8 @@
       <x:c r="DE4" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF4" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF4" s="115" t="str">
+        <x:v>#FFE6A6FF</x:v>
       </x:c>
       <x:c r="DG4" s="45" t="n">
         <x:v>60</x:v>
@@ -2401,8 +2587,8 @@
       <x:c r="DQ4" s="88"/>
       <x:c r="DR4" s="88"/>
       <x:c r="DS4" s="88"/>
-      <x:c r="DT4" s="100" t="n">
-        <x:v>3</x:v>
+      <x:c r="DT4" s="100" t="str">
+        <x:v>衝撃波</x:v>
       </x:c>
       <x:c r="DU4" s="106" t="str">
         <x:v>有効</x:v>
@@ -2413,6 +2599,7 @@
       <x:c r="DW4" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX4" s="109"/>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" s="9" t="str">
@@ -2739,8 +2926,8 @@
       <x:c r="DE5" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF5" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF5" s="117" t="str">
+        <x:v>#FFBE55FF</x:v>
       </x:c>
       <x:c r="DG5" s="45" t="n">
         <x:v>60</x:v>
@@ -2769,8 +2956,8 @@
       <x:c r="DQ5" s="88"/>
       <x:c r="DR5" s="88"/>
       <x:c r="DS5" s="88"/>
-      <x:c r="DT5" s="100" t="n">
-        <x:v>4</x:v>
+      <x:c r="DT5" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU5" s="106" t="str">
         <x:v>有効</x:v>
@@ -2781,6 +2968,7 @@
       <x:c r="DW5" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX5" s="109"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="9" t="str">
@@ -3107,8 +3295,8 @@
       <x:c r="DE6" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF6" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF6" s="119" t="str">
+        <x:v>#8EEDCFFF</x:v>
       </x:c>
       <x:c r="DG6" s="45" t="n">
         <x:v>60</x:v>
@@ -3137,8 +3325,8 @@
       <x:c r="DQ6" s="88"/>
       <x:c r="DR6" s="88"/>
       <x:c r="DS6" s="88"/>
-      <x:c r="DT6" s="100" t="n">
-        <x:v>5</x:v>
+      <x:c r="DT6" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU6" s="106" t="str">
         <x:v>有効</x:v>
@@ -3149,6 +3337,7 @@
       <x:c r="DW6" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX6" s="109"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="9" t="str">
@@ -3475,8 +3664,8 @@
       <x:c r="DE7" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF7" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF7" s="121" t="str">
+        <x:v>#E3A15CFF</x:v>
       </x:c>
       <x:c r="DG7" s="45" t="n">
         <x:v>60</x:v>
@@ -3505,8 +3694,8 @@
       <x:c r="DQ7" s="88"/>
       <x:c r="DR7" s="88"/>
       <x:c r="DS7" s="88"/>
-      <x:c r="DT7" s="100" t="n">
-        <x:v>6</x:v>
+      <x:c r="DT7" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU7" s="106" t="str">
         <x:v>有効</x:v>
@@ -3517,6 +3706,7 @@
       <x:c r="DW7" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX7" s="109"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="9" t="str">
@@ -3843,8 +4033,8 @@
       <x:c r="DE8" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF8" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF8" s="123" t="str">
+        <x:v>#B492FFB3</x:v>
       </x:c>
       <x:c r="DG8" s="45" t="n">
         <x:v>60</x:v>
@@ -3873,8 +4063,8 @@
       <x:c r="DQ8" s="88"/>
       <x:c r="DR8" s="88"/>
       <x:c r="DS8" s="88"/>
-      <x:c r="DT8" s="100" t="n">
-        <x:v>7</x:v>
+      <x:c r="DT8" s="100" t="str">
+        <x:v>魔方陣</x:v>
       </x:c>
       <x:c r="DU8" s="106" t="str">
         <x:v>有効</x:v>
@@ -3885,6 +4075,7 @@
       <x:c r="DW8" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX8" s="109"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="9" t="str">
@@ -4211,8 +4402,8 @@
       <x:c r="DE9" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF9" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF9" s="125" t="str">
+        <x:v>#9DFF57FF</x:v>
       </x:c>
       <x:c r="DG9" s="45" t="n">
         <x:v>60</x:v>
@@ -4241,8 +4432,8 @@
       <x:c r="DQ9" s="88"/>
       <x:c r="DR9" s="88"/>
       <x:c r="DS9" s="88"/>
-      <x:c r="DT9" s="100" t="n">
-        <x:v>8</x:v>
+      <x:c r="DT9" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU9" s="106" t="str">
         <x:v>有効</x:v>
@@ -4253,6 +4444,7 @@
       <x:c r="DW9" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX9" s="109"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="9" t="str">
@@ -4579,8 +4771,8 @@
       <x:c r="DE10" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF10" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF10" s="127" t="str">
+        <x:v>#FF5030FF</x:v>
       </x:c>
       <x:c r="DG10" s="45" t="n">
         <x:v>60</x:v>
@@ -4609,8 +4801,8 @@
       <x:c r="DQ10" s="88"/>
       <x:c r="DR10" s="88"/>
       <x:c r="DS10" s="88"/>
-      <x:c r="DT10" s="100" t="n">
-        <x:v>9</x:v>
+      <x:c r="DT10" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU10" s="106" t="str">
         <x:v>有効</x:v>
@@ -4621,6 +4813,7 @@
       <x:c r="DW10" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX10" s="109"/>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="9" t="str">
@@ -4947,8 +5140,8 @@
       <x:c r="DE11" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF11" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF11" s="129" t="str">
+        <x:v>#72DBFFFF</x:v>
       </x:c>
       <x:c r="DG11" s="45" t="n">
         <x:v>60</x:v>
@@ -4977,8 +5170,8 @@
       <x:c r="DQ11" s="88"/>
       <x:c r="DR11" s="88"/>
       <x:c r="DS11" s="88"/>
-      <x:c r="DT11" s="100" t="n">
-        <x:v>10</x:v>
+      <x:c r="DT11" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU11" s="106" t="str">
         <x:v>有効</x:v>
@@ -4989,6 +5182,7 @@
       <x:c r="DW11" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX11" s="109"/>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="9" t="str">
@@ -5315,8 +5509,8 @@
       <x:c r="DE12" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF12" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF12" s="131" t="str">
+        <x:v>#C18AFFCC</x:v>
       </x:c>
       <x:c r="DG12" s="45" t="n">
         <x:v>60</x:v>
@@ -5345,8 +5539,8 @@
       <x:c r="DQ12" s="88"/>
       <x:c r="DR12" s="88"/>
       <x:c r="DS12" s="88"/>
-      <x:c r="DT12" s="100" t="n">
-        <x:v>11</x:v>
+      <x:c r="DT12" s="100" t="str">
+        <x:v>魔方陣</x:v>
       </x:c>
       <x:c r="DU12" s="106" t="str">
         <x:v>有効</x:v>
@@ -5357,6 +5551,7 @@
       <x:c r="DW12" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX12" s="109"/>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="9" t="str">
@@ -5683,8 +5878,8 @@
       <x:c r="DE13" s="45" t="n">
         <x:v>0.3</x:v>
       </x:c>
-      <x:c r="DF13" s="77" t="str">
-        <x:v>#FFFFFFFF</x:v>
+      <x:c r="DF13" s="133" t="str">
+        <x:v>#BD70FFFF</x:v>
       </x:c>
       <x:c r="DG13" s="45" t="n">
         <x:v>60</x:v>
@@ -5713,8 +5908,8 @@
       <x:c r="DQ13" s="88"/>
       <x:c r="DR13" s="88"/>
       <x:c r="DS13" s="88"/>
-      <x:c r="DT13" s="100" t="n">
-        <x:v>12</x:v>
+      <x:c r="DT13" s="100" t="str">
+        <x:v>光の弾</x:v>
       </x:c>
       <x:c r="DU13" s="106" t="str">
         <x:v>有効</x:v>
@@ -5725,6 +5920,7 @@
       <x:c r="DW13" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX13" s="109"/>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="10" t="str">
@@ -5890,6 +6086,7 @@
       <x:c r="DU14" s="106"/>
       <x:c r="DV14" s="106"/>
       <x:c r="DW14" s="106"/>
+      <x:c r="DX14" s="109"/>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="10" t="str">
@@ -6055,6 +6252,7 @@
       <x:c r="DU15" s="106"/>
       <x:c r="DV15" s="106"/>
       <x:c r="DW15" s="106"/>
+      <x:c r="DX15" s="109"/>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="10" t="str">
@@ -6220,6 +6418,7 @@
       <x:c r="DU16" s="106"/>
       <x:c r="DV16" s="106"/>
       <x:c r="DW16" s="106"/>
+      <x:c r="DX16" s="109"/>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="10" t="str">
@@ -6385,6 +6584,7 @@
       <x:c r="DU17" s="106"/>
       <x:c r="DV17" s="106"/>
       <x:c r="DW17" s="106"/>
+      <x:c r="DX17" s="109"/>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="10" t="str">
@@ -6550,6 +6750,7 @@
       <x:c r="DU18" s="106"/>
       <x:c r="DV18" s="106"/>
       <x:c r="DW18" s="106"/>
+      <x:c r="DX18" s="109"/>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="10" t="str">
@@ -6715,6 +6916,7 @@
       <x:c r="DU19" s="106"/>
       <x:c r="DV19" s="106"/>
       <x:c r="DW19" s="106"/>
+      <x:c r="DX19" s="109"/>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="10" t="str">
@@ -6880,6 +7082,7 @@
       <x:c r="DU20" s="106"/>
       <x:c r="DV20" s="106"/>
       <x:c r="DW20" s="106"/>
+      <x:c r="DX20" s="109"/>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="10" t="str">
@@ -7045,6 +7248,7 @@
       <x:c r="DU21" s="106"/>
       <x:c r="DV21" s="106"/>
       <x:c r="DW21" s="106"/>
+      <x:c r="DX21" s="109"/>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="10" t="str">
@@ -7210,6 +7414,7 @@
       <x:c r="DU22" s="106"/>
       <x:c r="DV22" s="106"/>
       <x:c r="DW22" s="106"/>
+      <x:c r="DX22" s="109"/>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="10" t="str">
@@ -7375,6 +7580,7 @@
       <x:c r="DU23" s="106"/>
       <x:c r="DV23" s="106"/>
       <x:c r="DW23" s="106"/>
+      <x:c r="DX23" s="109"/>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="10" t="str">
@@ -7540,6 +7746,7 @@
       <x:c r="DU24" s="106"/>
       <x:c r="DV24" s="106"/>
       <x:c r="DW24" s="106"/>
+      <x:c r="DX24" s="109"/>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="10" t="str">
@@ -7705,6 +7912,7 @@
       <x:c r="DU25" s="106"/>
       <x:c r="DV25" s="106"/>
       <x:c r="DW25" s="106"/>
+      <x:c r="DX25" s="109"/>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="10" t="str">
@@ -7870,6 +8078,7 @@
       <x:c r="DU26" s="106"/>
       <x:c r="DV26" s="106"/>
       <x:c r="DW26" s="106"/>
+      <x:c r="DX26" s="109"/>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="10" t="str">
@@ -8035,6 +8244,7 @@
       <x:c r="DU27" s="106"/>
       <x:c r="DV27" s="106"/>
       <x:c r="DW27" s="106"/>
+      <x:c r="DX27" s="109"/>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="10" t="str">
@@ -8200,6 +8410,7 @@
       <x:c r="DU28" s="106"/>
       <x:c r="DV28" s="106"/>
       <x:c r="DW28" s="106"/>
+      <x:c r="DX28" s="109"/>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="10" t="str">
@@ -8365,6 +8576,7 @@
       <x:c r="DU29" s="106"/>
       <x:c r="DV29" s="106"/>
       <x:c r="DW29" s="106"/>
+      <x:c r="DX29" s="109"/>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="10" t="str">
@@ -8530,6 +8742,7 @@
       <x:c r="DU30" s="106"/>
       <x:c r="DV30" s="106"/>
       <x:c r="DW30" s="106"/>
+      <x:c r="DX30" s="109"/>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="10" t="str">
@@ -8695,6 +8908,7 @@
       <x:c r="DU31" s="106"/>
       <x:c r="DV31" s="106"/>
       <x:c r="DW31" s="106"/>
+      <x:c r="DX31" s="109"/>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
       <x:c r="A32" s="10" t="str">
@@ -8860,6 +9074,7 @@
       <x:c r="DU32" s="106"/>
       <x:c r="DV32" s="106"/>
       <x:c r="DW32" s="106"/>
+      <x:c r="DX32" s="109"/>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
       <x:c r="A33" s="10" t="str">
@@ -9025,6 +9240,7 @@
       <x:c r="DU33" s="106"/>
       <x:c r="DV33" s="106"/>
       <x:c r="DW33" s="106"/>
+      <x:c r="DX33" s="109"/>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
       <x:c r="A34" s="10" t="str">
@@ -9190,6 +9406,7 @@
       <x:c r="DU34" s="106"/>
       <x:c r="DV34" s="106"/>
       <x:c r="DW34" s="106"/>
+      <x:c r="DX34" s="109"/>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
       <x:c r="A35" s="10" t="str">
@@ -9355,6 +9572,7 @@
       <x:c r="DU35" s="106"/>
       <x:c r="DV35" s="106"/>
       <x:c r="DW35" s="106"/>
+      <x:c r="DX35" s="109"/>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
       <x:c r="A36" s="10" t="str">
@@ -9520,6 +9738,7 @@
       <x:c r="DU36" s="106"/>
       <x:c r="DV36" s="106"/>
       <x:c r="DW36" s="106"/>
+      <x:c r="DX36" s="109"/>
     </x:row>
     <x:row r="37" ht="25" customHeight="1">
       <x:c r="A37" s="10" t="str">
@@ -9685,6 +9904,7 @@
       <x:c r="DU37" s="106"/>
       <x:c r="DV37" s="106"/>
       <x:c r="DW37" s="106"/>
+      <x:c r="DX37" s="109"/>
     </x:row>
     <x:row r="38" ht="25" customHeight="1">
       <x:c r="A38" s="10" t="str">
@@ -9850,6 +10070,7 @@
       <x:c r="DU38" s="106"/>
       <x:c r="DV38" s="106"/>
       <x:c r="DW38" s="106"/>
+      <x:c r="DX38" s="109"/>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
       <x:c r="A39" s="10" t="str">
@@ -10015,6 +10236,7 @@
       <x:c r="DU39" s="106"/>
       <x:c r="DV39" s="106"/>
       <x:c r="DW39" s="106"/>
+      <x:c r="DX39" s="109"/>
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
       <x:c r="A40" s="93" t="str">
@@ -10341,8 +10563,8 @@
       <x:c r="DE40" s="90" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="DF40" s="90" t="str">
-        <x:v>#B4ECFFFF</x:v>
+      <x:c r="DF40" s="135" t="str">
+        <x:v>#FFE6A6FF</x:v>
       </x:c>
       <x:c r="DG40" s="90" t="n">
         <x:v>60</x:v>
@@ -10383,8 +10605,8 @@
       <x:c r="DS40" s="88" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="DT40" s="100" t="n">
-        <x:v>3</x:v>
+      <x:c r="DT40" s="100" t="str">
+        <x:v>衝撃波</x:v>
       </x:c>
       <x:c r="DU40" s="106" t="str">
         <x:v>有効</x:v>
@@ -10395,6 +10617,7 @@
       <x:c r="DW40" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX40" s="109"/>
     </x:row>
     <x:row r="41" ht="25" customHeight="1">
       <x:c r="A41" s="93" t="str">
@@ -10721,8 +10944,8 @@
       <x:c r="DE41" s="90" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="DF41" s="90" t="str">
-        <x:v>#FFAA66FF</x:v>
+      <x:c r="DF41" s="137" t="str">
+        <x:v>#FF6B38CC</x:v>
       </x:c>
       <x:c r="DG41" s="90" t="n">
         <x:v>60</x:v>
@@ -10763,8 +10986,8 @@
       <x:c r="DS41" s="88" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="DT41" s="100" t="n">
-        <x:v>7</x:v>
+      <x:c r="DT41" s="100" t="str">
+        <x:v>魔方陣</x:v>
       </x:c>
       <x:c r="DU41" s="106" t="str">
         <x:v>有効</x:v>
@@ -10775,6 +10998,7 @@
       <x:c r="DW41" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX41" s="109"/>
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
       <x:c r="A42" s="93" t="str">
@@ -11101,8 +11325,8 @@
       <x:c r="DE42" s="90" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="DF42" s="90" t="str">
-        <x:v>#8AFFBFFF</x:v>
+      <x:c r="DF42" s="139" t="str">
+        <x:v>#70FFACB3</x:v>
       </x:c>
       <x:c r="DG42" s="90" t="n">
         <x:v>60</x:v>
@@ -11143,8 +11367,8 @@
       <x:c r="DS42" s="88" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="DT42" s="100" t="n">
-        <x:v>2</x:v>
+      <x:c r="DT42" s="100" t="str">
+        <x:v>魔方陣</x:v>
       </x:c>
       <x:c r="DU42" s="106" t="str">
         <x:v>有効</x:v>
@@ -11155,6 +11379,7 @@
       <x:c r="DW42" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX42" s="109"/>
     </x:row>
     <x:row r="43" ht="25" customHeight="1">
       <x:c r="A43" s="93" t="str">
@@ -11481,8 +11706,8 @@
       <x:c r="DE43" s="90" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="DF43" s="90" t="str">
-        <x:v>#BDA8FFFF</x:v>
+      <x:c r="DF43" s="141" t="str">
+        <x:v>#83BCFFB3</x:v>
       </x:c>
       <x:c r="DG43" s="90" t="n">
         <x:v>60</x:v>
@@ -11523,8 +11748,8 @@
       <x:c r="DS43" s="88" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="DT43" s="100" t="n">
-        <x:v>4</x:v>
+      <x:c r="DT43" s="100" t="str">
+        <x:v>魔方陣</x:v>
       </x:c>
       <x:c r="DU43" s="106" t="str">
         <x:v>有効</x:v>
@@ -11535,6 +11760,7 @@
       <x:c r="DW43" s="106" t="n">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="DX43" s="109"/>
     </x:row>
     <x:row r="44" ht="25" customHeight="1">
       <x:c r="A44" s="10"/>
@@ -11624,6 +11850,7 @@
       <x:c r="DU44" s="106"/>
       <x:c r="DV44" s="106"/>
       <x:c r="DW44" s="106"/>
+      <x:c r="DX44" s="109"/>
     </x:row>
     <x:row r="45" ht="25" customHeight="1">
       <x:c r="A45" s="10"/>
@@ -11713,6 +11940,7 @@
       <x:c r="DU45" s="106"/>
       <x:c r="DV45" s="106"/>
       <x:c r="DW45" s="106"/>
+      <x:c r="DX45" s="109"/>
     </x:row>
     <x:row r="46" ht="25" customHeight="1">
       <x:c r="A46" s="10"/>
@@ -11802,6 +12030,7 @@
       <x:c r="DU46" s="106"/>
       <x:c r="DV46" s="106"/>
       <x:c r="DW46" s="106"/>
+      <x:c r="DX46" s="109"/>
     </x:row>
     <x:row r="47" ht="25" customHeight="1">
       <x:c r="A47" s="10"/>
@@ -11891,6 +12120,7 @@
       <x:c r="DU47" s="106"/>
       <x:c r="DV47" s="106"/>
       <x:c r="DW47" s="106"/>
+      <x:c r="DX47" s="109"/>
     </x:row>
     <x:row r="48" ht="25" customHeight="1">
       <x:c r="A48" s="10"/>
@@ -11980,6 +12210,7 @@
       <x:c r="DU48" s="106"/>
       <x:c r="DV48" s="106"/>
       <x:c r="DW48" s="106"/>
+      <x:c r="DX48" s="109"/>
     </x:row>
     <x:row r="49" ht="25" customHeight="1">
       <x:c r="A49" s="10"/>
@@ -12069,6 +12300,7 @@
       <x:c r="DU49" s="106"/>
       <x:c r="DV49" s="106"/>
       <x:c r="DW49" s="106"/>
+      <x:c r="DX49" s="109"/>
     </x:row>
     <x:row r="50" ht="25" customHeight="1">
       <x:c r="A50" s="10"/>
@@ -12158,6 +12390,7 @@
       <x:c r="DU50" s="106"/>
       <x:c r="DV50" s="106"/>
       <x:c r="DW50" s="106"/>
+      <x:c r="DX50" s="109"/>
     </x:row>
     <x:row r="51" ht="25" customHeight="1">
       <x:c r="A51" s="10"/>
@@ -12247,6 +12480,7 @@
       <x:c r="DU51" s="106"/>
       <x:c r="DV51" s="106"/>
       <x:c r="DW51" s="106"/>
+      <x:c r="DX51" s="109"/>
     </x:row>
     <x:row r="52" ht="25" customHeight="1">
       <x:c r="A52" s="10"/>
@@ -12336,6 +12570,7 @@
       <x:c r="DU52" s="106"/>
       <x:c r="DV52" s="106"/>
       <x:c r="DW52" s="106"/>
+      <x:c r="DX52" s="109"/>
     </x:row>
     <x:row r="53" ht="25" customHeight="1">
       <x:c r="A53" s="10"/>
@@ -12425,6 +12660,7 @@
       <x:c r="DU53" s="106"/>
       <x:c r="DV53" s="106"/>
       <x:c r="DW53" s="106"/>
+      <x:c r="DX53" s="109"/>
     </x:row>
     <x:row r="54" ht="25" customHeight="1">
       <x:c r="A54" s="10"/>
@@ -12514,6 +12750,7 @@
       <x:c r="DU54" s="106"/>
       <x:c r="DV54" s="106"/>
       <x:c r="DW54" s="106"/>
+      <x:c r="DX54" s="109"/>
     </x:row>
     <x:row r="55" ht="25" customHeight="1">
       <x:c r="A55" s="10"/>
@@ -12603,6 +12840,7 @@
       <x:c r="DU55" s="106"/>
       <x:c r="DV55" s="106"/>
       <x:c r="DW55" s="106"/>
+      <x:c r="DX55" s="109"/>
     </x:row>
     <x:row r="56" ht="25" customHeight="1">
       <x:c r="A56" s="10"/>
@@ -12692,6 +12930,7 @@
       <x:c r="DU56" s="106"/>
       <x:c r="DV56" s="106"/>
       <x:c r="DW56" s="106"/>
+      <x:c r="DX56" s="109"/>
     </x:row>
     <x:row r="57" ht="25" customHeight="1">
       <x:c r="A57" s="10"/>
@@ -12781,6 +13020,7 @@
       <x:c r="DU57" s="106"/>
       <x:c r="DV57" s="106"/>
       <x:c r="DW57" s="106"/>
+      <x:c r="DX57" s="109"/>
     </x:row>
     <x:row r="58" ht="25" customHeight="1">
       <x:c r="A58" s="10"/>
@@ -12870,6 +13110,7 @@
       <x:c r="DU58" s="106"/>
       <x:c r="DV58" s="106"/>
       <x:c r="DW58" s="106"/>
+      <x:c r="DX58" s="109"/>
     </x:row>
     <x:row r="59" ht="25" customHeight="1">
       <x:c r="A59" s="10"/>
@@ -12959,6 +13200,7 @@
       <x:c r="DU59" s="106"/>
       <x:c r="DV59" s="106"/>
       <x:c r="DW59" s="106"/>
+      <x:c r="DX59" s="109"/>
     </x:row>
     <x:row r="60" ht="25" customHeight="1">
       <x:c r="A60" s="10"/>
@@ -13048,6 +13290,7 @@
       <x:c r="DU60" s="106"/>
       <x:c r="DV60" s="106"/>
       <x:c r="DW60" s="106"/>
+      <x:c r="DX60" s="109"/>
     </x:row>
     <x:row r="61" ht="25" customHeight="1">
       <x:c r="A61" s="10"/>
@@ -13137,6 +13380,7 @@
       <x:c r="DU61" s="106"/>
       <x:c r="DV61" s="106"/>
       <x:c r="DW61" s="106"/>
+      <x:c r="DX61" s="109"/>
     </x:row>
     <x:row r="62" ht="25" customHeight="1">
       <x:c r="A62" s="10"/>
@@ -13226,6 +13470,7 @@
       <x:c r="DU62" s="106"/>
       <x:c r="DV62" s="106"/>
       <x:c r="DW62" s="106"/>
+      <x:c r="DX62" s="109"/>
     </x:row>
     <x:row r="63" ht="25" customHeight="1">
       <x:c r="A63" s="10"/>
@@ -13315,6 +13560,7 @@
       <x:c r="DU63" s="106"/>
       <x:c r="DV63" s="106"/>
       <x:c r="DW63" s="106"/>
+      <x:c r="DX63" s="109"/>
     </x:row>
     <x:row r="64" ht="25" customHeight="1">
       <x:c r="A64" s="10"/>
@@ -13404,6 +13650,7 @@
       <x:c r="DU64" s="106"/>
       <x:c r="DV64" s="106"/>
       <x:c r="DW64" s="106"/>
+      <x:c r="DX64" s="109"/>
     </x:row>
     <x:row r="65" ht="25" customHeight="1">
       <x:c r="A65" s="10"/>
@@ -13493,6 +13740,7 @@
       <x:c r="DU65" s="106"/>
       <x:c r="DV65" s="106"/>
       <x:c r="DW65" s="106"/>
+      <x:c r="DX65" s="109"/>
     </x:row>
     <x:row r="66" ht="25" customHeight="1">
       <x:c r="A66" s="10"/>
@@ -13582,6 +13830,7 @@
       <x:c r="DU66" s="106"/>
       <x:c r="DV66" s="106"/>
       <x:c r="DW66" s="106"/>
+      <x:c r="DX66" s="109"/>
     </x:row>
     <x:row r="67" ht="25" customHeight="1">
       <x:c r="A67" s="10"/>
@@ -13671,6 +13920,7 @@
       <x:c r="DU67" s="106"/>
       <x:c r="DV67" s="106"/>
       <x:c r="DW67" s="106"/>
+      <x:c r="DX67" s="109"/>
     </x:row>
     <x:row r="68" ht="25" customHeight="1">
       <x:c r="A68" s="10"/>
@@ -13760,6 +14010,7 @@
       <x:c r="DU68" s="106"/>
       <x:c r="DV68" s="106"/>
       <x:c r="DW68" s="106"/>
+      <x:c r="DX68" s="109"/>
     </x:row>
     <x:row r="69" ht="25" customHeight="1">
       <x:c r="A69" s="10"/>
@@ -13849,6 +14100,7 @@
       <x:c r="DU69" s="106"/>
       <x:c r="DV69" s="106"/>
       <x:c r="DW69" s="106"/>
+      <x:c r="DX69" s="109"/>
     </x:row>
     <x:row r="70" ht="25" customHeight="1">
       <x:c r="A70" s="10"/>
@@ -13938,6 +14190,7 @@
       <x:c r="DU70" s="106"/>
       <x:c r="DV70" s="106"/>
       <x:c r="DW70" s="106"/>
+      <x:c r="DX70" s="109"/>
     </x:row>
     <x:row r="71" ht="25" customHeight="1">
       <x:c r="A71" s="10"/>
@@ -14027,6 +14280,7 @@
       <x:c r="DU71" s="106"/>
       <x:c r="DV71" s="106"/>
       <x:c r="DW71" s="106"/>
+      <x:c r="DX71" s="109"/>
     </x:row>
     <x:row r="72" ht="25" customHeight="1">
       <x:c r="A72" s="10"/>
@@ -14116,6 +14370,7 @@
       <x:c r="DU72" s="106"/>
       <x:c r="DV72" s="106"/>
       <x:c r="DW72" s="106"/>
+      <x:c r="DX72" s="109"/>
     </x:row>
     <x:row r="73" ht="25" customHeight="1">
       <x:c r="A73" s="10"/>
@@ -14205,6 +14460,7 @@
       <x:c r="DU73" s="106"/>
       <x:c r="DV73" s="106"/>
       <x:c r="DW73" s="106"/>
+      <x:c r="DX73" s="109"/>
     </x:row>
     <x:row r="74" ht="25" customHeight="1">
       <x:c r="A74" s="10"/>
@@ -14294,6 +14550,7 @@
       <x:c r="DU74" s="106"/>
       <x:c r="DV74" s="106"/>
       <x:c r="DW74" s="106"/>
+      <x:c r="DX74" s="109"/>
     </x:row>
     <x:row r="75" ht="25" customHeight="1">
       <x:c r="A75" s="10"/>
@@ -14383,6 +14640,7 @@
       <x:c r="DU75" s="106"/>
       <x:c r="DV75" s="106"/>
       <x:c r="DW75" s="106"/>
+      <x:c r="DX75" s="109"/>
     </x:row>
     <x:row r="76" ht="25" customHeight="1">
       <x:c r="A76" s="10"/>
@@ -14472,6 +14730,7 @@
       <x:c r="DU76" s="106"/>
       <x:c r="DV76" s="106"/>
       <x:c r="DW76" s="106"/>
+      <x:c r="DX76" s="109"/>
     </x:row>
     <x:row r="77" ht="25" customHeight="1">
       <x:c r="A77" s="10"/>
@@ -14561,6 +14820,7 @@
       <x:c r="DU77" s="106"/>
       <x:c r="DV77" s="106"/>
       <x:c r="DW77" s="106"/>
+      <x:c r="DX77" s="109"/>
     </x:row>
     <x:row r="78" ht="25" customHeight="1">
       <x:c r="A78" s="10"/>
@@ -14650,6 +14910,7 @@
       <x:c r="DU78" s="106"/>
       <x:c r="DV78" s="106"/>
       <x:c r="DW78" s="106"/>
+      <x:c r="DX78" s="109"/>
     </x:row>
     <x:row r="79" ht="25" customHeight="1">
       <x:c r="A79" s="10"/>
@@ -14739,6 +15000,7 @@
       <x:c r="DU79" s="106"/>
       <x:c r="DV79" s="106"/>
       <x:c r="DW79" s="106"/>
+      <x:c r="DX79" s="109"/>
     </x:row>
     <x:row r="80" ht="25" customHeight="1">
       <x:c r="A80" s="10"/>
@@ -14828,6 +15090,7 @@
       <x:c r="DU80" s="106"/>
       <x:c r="DV80" s="106"/>
       <x:c r="DW80" s="106"/>
+      <x:c r="DX80" s="109"/>
     </x:row>
     <x:row r="81" ht="25" customHeight="1">
       <x:c r="A81" s="10"/>
@@ -14917,6 +15180,7 @@
       <x:c r="DU81" s="106"/>
       <x:c r="DV81" s="106"/>
       <x:c r="DW81" s="106"/>
+      <x:c r="DX81" s="109"/>
     </x:row>
     <x:row r="82" ht="25" customHeight="1">
       <x:c r="A82" s="10"/>
@@ -15006,6 +15270,7 @@
       <x:c r="DU82" s="106"/>
       <x:c r="DV82" s="106"/>
       <x:c r="DW82" s="106"/>
+      <x:c r="DX82" s="109"/>
     </x:row>
     <x:row r="83" ht="25" customHeight="1">
       <x:c r="A83" s="10"/>
@@ -15095,6 +15360,7 @@
       <x:c r="DU83" s="106"/>
       <x:c r="DV83" s="106"/>
       <x:c r="DW83" s="106"/>
+      <x:c r="DX83" s="109"/>
     </x:row>
     <x:row r="84" ht="25" customHeight="1">
       <x:c r="A84" s="10"/>
@@ -15184,6 +15450,7 @@
       <x:c r="DU84" s="106"/>
       <x:c r="DV84" s="106"/>
       <x:c r="DW84" s="106"/>
+      <x:c r="DX84" s="109"/>
     </x:row>
     <x:row r="85" ht="25" customHeight="1">
       <x:c r="A85" s="10"/>
@@ -15273,6 +15540,7 @@
       <x:c r="DU85" s="106"/>
       <x:c r="DV85" s="106"/>
       <x:c r="DW85" s="106"/>
+      <x:c r="DX85" s="109"/>
     </x:row>
     <x:row r="86" ht="25" customHeight="1">
       <x:c r="A86" s="10"/>
@@ -15362,6 +15630,7 @@
       <x:c r="DU86" s="106"/>
       <x:c r="DV86" s="106"/>
       <x:c r="DW86" s="106"/>
+      <x:c r="DX86" s="109"/>
     </x:row>
     <x:row r="87" ht="25" customHeight="1">
       <x:c r="A87" s="10"/>
@@ -15451,6 +15720,7 @@
       <x:c r="DU87" s="106"/>
       <x:c r="DV87" s="106"/>
       <x:c r="DW87" s="106"/>
+      <x:c r="DX87" s="109"/>
     </x:row>
     <x:row r="88" ht="25" customHeight="1">
       <x:c r="A88" s="10"/>
@@ -15540,6 +15810,7 @@
       <x:c r="DU88" s="106"/>
       <x:c r="DV88" s="106"/>
       <x:c r="DW88" s="106"/>
+      <x:c r="DX88" s="109"/>
     </x:row>
     <x:row r="89" ht="25" customHeight="1">
       <x:c r="A89" s="10"/>
@@ -15629,6 +15900,7 @@
       <x:c r="DU89" s="106"/>
       <x:c r="DV89" s="106"/>
       <x:c r="DW89" s="106"/>
+      <x:c r="DX89" s="109"/>
     </x:row>
     <x:row r="90" ht="25" customHeight="1">
       <x:c r="A90" s="10"/>
@@ -15718,6 +15990,7 @@
       <x:c r="DU90" s="106"/>
       <x:c r="DV90" s="106"/>
       <x:c r="DW90" s="106"/>
+      <x:c r="DX90" s="109"/>
     </x:row>
     <x:row r="91" ht="25" customHeight="1">
       <x:c r="A91" s="10"/>
@@ -15807,6 +16080,7 @@
       <x:c r="DU91" s="106"/>
       <x:c r="DV91" s="106"/>
       <x:c r="DW91" s="106"/>
+      <x:c r="DX91" s="109"/>
     </x:row>
     <x:row r="92" ht="25" customHeight="1">
       <x:c r="A92" s="10"/>
@@ -15896,6 +16170,7 @@
       <x:c r="DU92" s="106"/>
       <x:c r="DV92" s="106"/>
       <x:c r="DW92" s="106"/>
+      <x:c r="DX92" s="109"/>
     </x:row>
     <x:row r="93" ht="25" customHeight="1">
       <x:c r="A93" s="10"/>
@@ -15985,6 +16260,7 @@
       <x:c r="DU93" s="106"/>
       <x:c r="DV93" s="106"/>
       <x:c r="DW93" s="106"/>
+      <x:c r="DX93" s="109"/>
     </x:row>
     <x:row r="94" ht="25" customHeight="1">
       <x:c r="A94" s="10"/>
@@ -16074,6 +16350,7 @@
       <x:c r="DU94" s="106"/>
       <x:c r="DV94" s="106"/>
       <x:c r="DW94" s="106"/>
+      <x:c r="DX94" s="109"/>
     </x:row>
     <x:row r="95" ht="25" customHeight="1">
       <x:c r="A95" s="10"/>
@@ -16163,6 +16440,7 @@
       <x:c r="DU95" s="106"/>
       <x:c r="DV95" s="106"/>
       <x:c r="DW95" s="106"/>
+      <x:c r="DX95" s="109"/>
     </x:row>
     <x:row r="96" ht="25" customHeight="1">
       <x:c r="A96" s="10"/>
@@ -16252,6 +16530,7 @@
       <x:c r="DU96" s="106"/>
       <x:c r="DV96" s="106"/>
       <x:c r="DW96" s="106"/>
+      <x:c r="DX96" s="109"/>
     </x:row>
     <x:row r="97" ht="25" customHeight="1">
       <x:c r="A97" s="10"/>
@@ -16341,6 +16620,7 @@
       <x:c r="DU97" s="106"/>
       <x:c r="DV97" s="106"/>
       <x:c r="DW97" s="106"/>
+      <x:c r="DX97" s="109"/>
     </x:row>
     <x:row r="98" ht="25" customHeight="1">
       <x:c r="A98" s="10"/>
@@ -16430,6 +16710,7 @@
       <x:c r="DU98" s="106"/>
       <x:c r="DV98" s="106"/>
       <x:c r="DW98" s="106"/>
+      <x:c r="DX98" s="109"/>
     </x:row>
     <x:row r="99" ht="25" customHeight="1">
       <x:c r="A99" s="10"/>
@@ -16519,6 +16800,7 @@
       <x:c r="DU99" s="106"/>
       <x:c r="DV99" s="106"/>
       <x:c r="DW99" s="106"/>
+      <x:c r="DX99" s="109"/>
     </x:row>
     <x:row r="100" ht="25" customHeight="1">
       <x:c r="A100" s="10"/>
@@ -16608,6 +16890,7 @@
       <x:c r="DU100" s="106"/>
       <x:c r="DV100" s="106"/>
       <x:c r="DW100" s="106"/>
+      <x:c r="DX100" s="109"/>
     </x:row>
     <x:row r="101" ht="25" customHeight="1">
       <x:c r="A101" s="10"/>
@@ -16697,6 +16980,7 @@
       <x:c r="DU101" s="106"/>
       <x:c r="DV101" s="106"/>
       <x:c r="DW101" s="106"/>
+      <x:c r="DX101" s="109"/>
     </x:row>
     <x:row r="102" ht="25" customHeight="1">
       <x:c r="A102" s="10"/>
@@ -16786,6 +17070,7 @@
       <x:c r="DU102" s="106"/>
       <x:c r="DV102" s="106"/>
       <x:c r="DW102" s="106"/>
+      <x:c r="DX102" s="109"/>
     </x:row>
     <x:row r="103" ht="25" customHeight="1">
       <x:c r="A103" s="10"/>
@@ -16875,6 +17160,7 @@
       <x:c r="DU103" s="106"/>
       <x:c r="DV103" s="106"/>
       <x:c r="DW103" s="106"/>
+      <x:c r="DX103" s="109"/>
     </x:row>
     <x:row r="104" ht="25" customHeight="1">
       <x:c r="A104" s="10"/>
@@ -16964,6 +17250,7 @@
       <x:c r="DU104" s="106"/>
       <x:c r="DV104" s="106"/>
       <x:c r="DW104" s="106"/>
+      <x:c r="DX104" s="109"/>
     </x:row>
     <x:row r="105" ht="25" customHeight="1">
       <x:c r="A105" s="10"/>
@@ -17053,6 +17340,7 @@
       <x:c r="DU105" s="106"/>
       <x:c r="DV105" s="106"/>
       <x:c r="DW105" s="106"/>
+      <x:c r="DX105" s="109"/>
     </x:row>
     <x:row r="106" ht="25" customHeight="1">
       <x:c r="A106" s="10"/>
@@ -17142,6 +17430,7 @@
       <x:c r="DU106" s="106"/>
       <x:c r="DV106" s="106"/>
       <x:c r="DW106" s="106"/>
+      <x:c r="DX106" s="109"/>
     </x:row>
     <x:row r="107" ht="25" customHeight="1">
       <x:c r="A107" s="10"/>
@@ -17231,6 +17520,7 @@
       <x:c r="DU107" s="106"/>
       <x:c r="DV107" s="106"/>
       <x:c r="DW107" s="106"/>
+      <x:c r="DX107" s="109"/>
     </x:row>
     <x:row r="108" ht="25" customHeight="1">
       <x:c r="A108" s="10"/>
@@ -17320,6 +17610,7 @@
       <x:c r="DU108" s="106"/>
       <x:c r="DV108" s="106"/>
       <x:c r="DW108" s="106"/>
+      <x:c r="DX108" s="109"/>
     </x:row>
     <x:row r="109" ht="25" customHeight="1">
       <x:c r="A109" s="10"/>
@@ -17409,6 +17700,7 @@
       <x:c r="DU109" s="106"/>
       <x:c r="DV109" s="106"/>
       <x:c r="DW109" s="106"/>
+      <x:c r="DX109" s="109"/>
     </x:row>
     <x:row r="110" ht="25" customHeight="1">
       <x:c r="A110" s="10"/>
@@ -17498,6 +17790,7 @@
       <x:c r="DU110" s="106"/>
       <x:c r="DV110" s="106"/>
       <x:c r="DW110" s="106"/>
+      <x:c r="DX110" s="109"/>
     </x:row>
     <x:row r="111" ht="25" customHeight="1">
       <x:c r="A111" s="10"/>
@@ -17587,6 +17880,7 @@
       <x:c r="DU111" s="106"/>
       <x:c r="DV111" s="106"/>
       <x:c r="DW111" s="106"/>
+      <x:c r="DX111" s="109"/>
     </x:row>
     <x:row r="112" ht="25" customHeight="1">
       <x:c r="A112" s="10"/>
@@ -17676,6 +17970,7 @@
       <x:c r="DU112" s="106"/>
       <x:c r="DV112" s="106"/>
       <x:c r="DW112" s="106"/>
+      <x:c r="DX112" s="109"/>
     </x:row>
     <x:row r="113" ht="25" customHeight="1">
       <x:c r="A113" s="10"/>
@@ -17765,6 +18060,7 @@
       <x:c r="DU113" s="106"/>
       <x:c r="DV113" s="106"/>
       <x:c r="DW113" s="106"/>
+      <x:c r="DX113" s="109"/>
     </x:row>
     <x:row r="114" ht="25" customHeight="1">
       <x:c r="A114" s="10"/>
@@ -17854,6 +18150,7 @@
       <x:c r="DU114" s="106"/>
       <x:c r="DV114" s="106"/>
       <x:c r="DW114" s="106"/>
+      <x:c r="DX114" s="109"/>
     </x:row>
     <x:row r="115" ht="25" customHeight="1">
       <x:c r="A115" s="10"/>
@@ -17943,6 +18240,7 @@
       <x:c r="DU115" s="106"/>
       <x:c r="DV115" s="106"/>
       <x:c r="DW115" s="106"/>
+      <x:c r="DX115" s="109"/>
     </x:row>
     <x:row r="116" ht="25" customHeight="1">
       <x:c r="A116" s="10"/>
@@ -18032,6 +18330,7 @@
       <x:c r="DU116" s="106"/>
       <x:c r="DV116" s="106"/>
       <x:c r="DW116" s="106"/>
+      <x:c r="DX116" s="109"/>
     </x:row>
     <x:row r="117" ht="25" customHeight="1">
       <x:c r="A117" s="10"/>
@@ -18121,6 +18420,7 @@
       <x:c r="DU117" s="106"/>
       <x:c r="DV117" s="106"/>
       <x:c r="DW117" s="106"/>
+      <x:c r="DX117" s="109"/>
     </x:row>
     <x:row r="118" ht="25" customHeight="1">
       <x:c r="A118" s="10"/>
@@ -18210,6 +18510,7 @@
       <x:c r="DU118" s="106"/>
       <x:c r="DV118" s="106"/>
       <x:c r="DW118" s="106"/>
+      <x:c r="DX118" s="109"/>
     </x:row>
     <x:row r="119" ht="25" customHeight="1">
       <x:c r="A119" s="10"/>
@@ -18299,6 +18600,7 @@
       <x:c r="DU119" s="106"/>
       <x:c r="DV119" s="106"/>
       <x:c r="DW119" s="106"/>
+      <x:c r="DX119" s="109"/>
     </x:row>
     <x:row r="120" ht="25" customHeight="1">
       <x:c r="A120" s="10"/>
@@ -18388,6 +18690,7 @@
       <x:c r="DU120" s="106"/>
       <x:c r="DV120" s="106"/>
       <x:c r="DW120" s="106"/>
+      <x:c r="DX120" s="109"/>
     </x:row>
     <x:row r="121" ht="25" customHeight="1">
       <x:c r="A121" s="10"/>
@@ -18477,6 +18780,7 @@
       <x:c r="DU121" s="106"/>
       <x:c r="DV121" s="106"/>
       <x:c r="DW121" s="106"/>
+      <x:c r="DX121" s="109"/>
     </x:row>
     <x:row r="122" ht="25" customHeight="1">
       <x:c r="A122" s="10"/>
@@ -18566,6 +18870,7 @@
       <x:c r="DU122" s="106"/>
       <x:c r="DV122" s="106"/>
       <x:c r="DW122" s="106"/>
+      <x:c r="DX122" s="109"/>
     </x:row>
     <x:row r="123" ht="25" customHeight="1">
       <x:c r="A123" s="10"/>
@@ -18655,6 +18960,7 @@
       <x:c r="DU123" s="106"/>
       <x:c r="DV123" s="106"/>
       <x:c r="DW123" s="106"/>
+      <x:c r="DX123" s="109"/>
     </x:row>
     <x:row r="124" ht="25" customHeight="1">
       <x:c r="A124" s="10"/>
@@ -18744,6 +19050,7 @@
       <x:c r="DU124" s="106"/>
       <x:c r="DV124" s="106"/>
       <x:c r="DW124" s="106"/>
+      <x:c r="DX124" s="109"/>
     </x:row>
     <x:row r="125" ht="25" customHeight="1">
       <x:c r="A125" s="10"/>
@@ -18833,6 +19140,7 @@
       <x:c r="DU125" s="106"/>
       <x:c r="DV125" s="106"/>
       <x:c r="DW125" s="106"/>
+      <x:c r="DX125" s="109"/>
     </x:row>
     <x:row r="126" ht="25" customHeight="1">
       <x:c r="A126" s="10"/>
@@ -18922,6 +19230,7 @@
       <x:c r="DU126" s="106"/>
       <x:c r="DV126" s="106"/>
       <x:c r="DW126" s="106"/>
+      <x:c r="DX126" s="109"/>
     </x:row>
     <x:row r="127" ht="25" customHeight="1">
       <x:c r="A127" s="10"/>
@@ -19011,6 +19320,7 @@
       <x:c r="DU127" s="106"/>
       <x:c r="DV127" s="106"/>
       <x:c r="DW127" s="106"/>
+      <x:c r="DX127" s="109"/>
     </x:row>
     <x:row r="128" ht="25" customHeight="1">
       <x:c r="A128" s="10"/>
@@ -19100,6 +19410,7 @@
       <x:c r="DU128" s="106"/>
       <x:c r="DV128" s="106"/>
       <x:c r="DW128" s="106"/>
+      <x:c r="DX128" s="109"/>
     </x:row>
     <x:row r="129" ht="25" customHeight="1">
       <x:c r="A129" s="10"/>
@@ -19189,6 +19500,7 @@
       <x:c r="DU129" s="106"/>
       <x:c r="DV129" s="106"/>
       <x:c r="DW129" s="106"/>
+      <x:c r="DX129" s="109"/>
     </x:row>
     <x:row r="130" ht="25" customHeight="1">
       <x:c r="A130" s="10"/>
@@ -19278,6 +19590,7 @@
       <x:c r="DU130" s="106"/>
       <x:c r="DV130" s="106"/>
       <x:c r="DW130" s="106"/>
+      <x:c r="DX130" s="109"/>
     </x:row>
     <x:row r="131" ht="25" customHeight="1">
       <x:c r="A131" s="10"/>
@@ -19367,6 +19680,7 @@
       <x:c r="DU131" s="106"/>
       <x:c r="DV131" s="106"/>
       <x:c r="DW131" s="106"/>
+      <x:c r="DX131" s="109"/>
     </x:row>
     <x:row r="132" ht="25" customHeight="1">
       <x:c r="A132" s="10"/>
@@ -19456,6 +19770,7 @@
       <x:c r="DU132" s="106"/>
       <x:c r="DV132" s="106"/>
       <x:c r="DW132" s="106"/>
+      <x:c r="DX132" s="109"/>
     </x:row>
     <x:row r="133" ht="25" customHeight="1">
       <x:c r="A133" s="10"/>
@@ -19545,6 +19860,7 @@
       <x:c r="DU133" s="106"/>
       <x:c r="DV133" s="106"/>
       <x:c r="DW133" s="106"/>
+      <x:c r="DX133" s="109"/>
     </x:row>
     <x:row r="134" ht="25" customHeight="1">
       <x:c r="A134" s="10"/>
@@ -19634,6 +19950,7 @@
       <x:c r="DU134" s="106"/>
       <x:c r="DV134" s="106"/>
       <x:c r="DW134" s="106"/>
+      <x:c r="DX134" s="109"/>
     </x:row>
     <x:row r="135" ht="25" customHeight="1">
       <x:c r="A135" s="10"/>
@@ -19723,6 +20040,7 @@
       <x:c r="DU135" s="106"/>
       <x:c r="DV135" s="106"/>
       <x:c r="DW135" s="106"/>
+      <x:c r="DX135" s="109"/>
     </x:row>
     <x:row r="136" ht="25" customHeight="1">
       <x:c r="A136" s="10"/>
@@ -19812,6 +20130,7 @@
       <x:c r="DU136" s="106"/>
       <x:c r="DV136" s="106"/>
       <x:c r="DW136" s="106"/>
+      <x:c r="DX136" s="109"/>
     </x:row>
     <x:row r="137" ht="25" customHeight="1">
       <x:c r="A137" s="10"/>
@@ -19901,6 +20220,7 @@
       <x:c r="DU137" s="106"/>
       <x:c r="DV137" s="106"/>
       <x:c r="DW137" s="106"/>
+      <x:c r="DX137" s="109"/>
     </x:row>
     <x:row r="138" ht="25" customHeight="1">
       <x:c r="A138" s="10"/>
@@ -19990,6 +20310,7 @@
       <x:c r="DU138" s="106"/>
       <x:c r="DV138" s="106"/>
       <x:c r="DW138" s="106"/>
+      <x:c r="DX138" s="109"/>
     </x:row>
     <x:row r="139" ht="25" customHeight="1">
       <x:c r="A139" s="10"/>
@@ -20079,6 +20400,7 @@
       <x:c r="DU139" s="106"/>
       <x:c r="DV139" s="106"/>
       <x:c r="DW139" s="106"/>
+      <x:c r="DX139" s="109"/>
     </x:row>
     <x:row r="140" ht="25" customHeight="1">
       <x:c r="A140" s="10"/>
@@ -20168,6 +20490,7 @@
       <x:c r="DU140" s="106"/>
       <x:c r="DV140" s="106"/>
       <x:c r="DW140" s="106"/>
+      <x:c r="DX140" s="109"/>
     </x:row>
     <x:row r="141" ht="25" customHeight="1">
       <x:c r="A141" s="10"/>
@@ -20257,6 +20580,7 @@
       <x:c r="DU141" s="106"/>
       <x:c r="DV141" s="106"/>
       <x:c r="DW141" s="106"/>
+      <x:c r="DX141" s="109"/>
     </x:row>
     <x:row r="142" ht="25" customHeight="1">
       <x:c r="A142" s="10"/>
@@ -20346,6 +20670,7 @@
       <x:c r="DU142" s="106"/>
       <x:c r="DV142" s="106"/>
       <x:c r="DW142" s="106"/>
+      <x:c r="DX142" s="109"/>
     </x:row>
     <x:row r="143" ht="25" customHeight="1">
       <x:c r="A143" s="10"/>
@@ -20435,6 +20760,7 @@
       <x:c r="DU143" s="106"/>
       <x:c r="DV143" s="106"/>
       <x:c r="DW143" s="106"/>
+      <x:c r="DX143" s="109"/>
     </x:row>
     <x:row r="144" ht="25" customHeight="1">
       <x:c r="A144" s="10"/>
@@ -20524,6 +20850,7 @@
       <x:c r="DU144" s="106"/>
       <x:c r="DV144" s="106"/>
       <x:c r="DW144" s="106"/>
+      <x:c r="DX144" s="109"/>
     </x:row>
     <x:row r="145" ht="25" customHeight="1">
       <x:c r="A145" s="10"/>
@@ -20613,6 +20940,7 @@
       <x:c r="DU145" s="106"/>
       <x:c r="DV145" s="106"/>
       <x:c r="DW145" s="106"/>
+      <x:c r="DX145" s="109"/>
     </x:row>
     <x:row r="146" ht="25" customHeight="1">
       <x:c r="A146" s="10"/>
@@ -20702,6 +21030,7 @@
       <x:c r="DU146" s="106"/>
       <x:c r="DV146" s="106"/>
       <x:c r="DW146" s="106"/>
+      <x:c r="DX146" s="109"/>
     </x:row>
     <x:row r="147" ht="25" customHeight="1">
       <x:c r="A147" s="10"/>
@@ -20791,6 +21120,7 @@
       <x:c r="DU147" s="106"/>
       <x:c r="DV147" s="106"/>
       <x:c r="DW147" s="106"/>
+      <x:c r="DX147" s="109"/>
     </x:row>
     <x:row r="148" ht="25" customHeight="1">
       <x:c r="A148" s="10"/>
@@ -20880,6 +21210,7 @@
       <x:c r="DU148" s="106"/>
       <x:c r="DV148" s="106"/>
       <x:c r="DW148" s="106"/>
+      <x:c r="DX148" s="109"/>
     </x:row>
     <x:row r="149" ht="25" customHeight="1">
       <x:c r="A149" s="10"/>
@@ -20969,6 +21300,7 @@
       <x:c r="DU149" s="106"/>
       <x:c r="DV149" s="106"/>
       <x:c r="DW149" s="106"/>
+      <x:c r="DX149" s="109"/>
     </x:row>
     <x:row r="150" ht="25" customHeight="1">
       <x:c r="A150" s="10"/>
@@ -21058,6 +21390,7 @@
       <x:c r="DU150" s="106"/>
       <x:c r="DV150" s="106"/>
       <x:c r="DW150" s="106"/>
+      <x:c r="DX150" s="109"/>
     </x:row>
     <x:row r="151" ht="25" customHeight="1">
       <x:c r="A151" s="10"/>
@@ -21147,6 +21480,7 @@
       <x:c r="DU151" s="106"/>
       <x:c r="DV151" s="106"/>
       <x:c r="DW151" s="106"/>
+      <x:c r="DX151" s="109"/>
     </x:row>
     <x:row r="152" ht="25" customHeight="1">
       <x:c r="A152" s="10"/>
@@ -21236,6 +21570,7 @@
       <x:c r="DU152" s="106"/>
       <x:c r="DV152" s="106"/>
       <x:c r="DW152" s="106"/>
+      <x:c r="DX152" s="109"/>
     </x:row>
     <x:row r="153" ht="25" customHeight="1">
       <x:c r="A153" s="10"/>
@@ -21325,6 +21660,7 @@
       <x:c r="DU153" s="106"/>
       <x:c r="DV153" s="106"/>
       <x:c r="DW153" s="106"/>
+      <x:c r="DX153" s="109"/>
     </x:row>
     <x:row r="154" ht="25" customHeight="1">
       <x:c r="A154" s="10"/>
@@ -21414,6 +21750,7 @@
       <x:c r="DU154" s="106"/>
       <x:c r="DV154" s="106"/>
       <x:c r="DW154" s="106"/>
+      <x:c r="DX154" s="109"/>
     </x:row>
     <x:row r="155" ht="25" customHeight="1">
       <x:c r="A155" s="10"/>
@@ -21503,6 +21840,7 @@
       <x:c r="DU155" s="106"/>
       <x:c r="DV155" s="106"/>
       <x:c r="DW155" s="106"/>
+      <x:c r="DX155" s="109"/>
     </x:row>
     <x:row r="156" ht="25" customHeight="1">
       <x:c r="A156" s="10"/>
@@ -21592,6 +21930,7 @@
       <x:c r="DU156" s="106"/>
       <x:c r="DV156" s="106"/>
       <x:c r="DW156" s="106"/>
+      <x:c r="DX156" s="109"/>
     </x:row>
     <x:row r="157" ht="25" customHeight="1">
       <x:c r="A157" s="10"/>
@@ -21681,6 +22020,7 @@
       <x:c r="DU157" s="106"/>
       <x:c r="DV157" s="106"/>
       <x:c r="DW157" s="106"/>
+      <x:c r="DX157" s="109"/>
     </x:row>
     <x:row r="158" ht="25" customHeight="1">
       <x:c r="A158" s="10"/>
@@ -21770,6 +22110,7 @@
       <x:c r="DU158" s="106"/>
       <x:c r="DV158" s="106"/>
       <x:c r="DW158" s="106"/>
+      <x:c r="DX158" s="109"/>
     </x:row>
     <x:row r="159" ht="25" customHeight="1">
       <x:c r="A159" s="10"/>
@@ -21859,6 +22200,7 @@
       <x:c r="DU159" s="106"/>
       <x:c r="DV159" s="106"/>
       <x:c r="DW159" s="106"/>
+      <x:c r="DX159" s="109"/>
     </x:row>
     <x:row r="160" ht="25" customHeight="1">
       <x:c r="A160" s="10"/>
@@ -21948,6 +22290,7 @@
       <x:c r="DU160" s="106"/>
       <x:c r="DV160" s="106"/>
       <x:c r="DW160" s="106"/>
+      <x:c r="DX160" s="109"/>
     </x:row>
     <x:row r="161" ht="25" customHeight="1">
       <x:c r="A161" s="10"/>
@@ -22037,6 +22380,7 @@
       <x:c r="DU161" s="106"/>
       <x:c r="DV161" s="106"/>
       <x:c r="DW161" s="106"/>
+      <x:c r="DX161" s="109"/>
     </x:row>
     <x:row r="162" ht="25" customHeight="1">
       <x:c r="A162" s="10"/>
@@ -22126,6 +22470,7 @@
       <x:c r="DU162" s="106"/>
       <x:c r="DV162" s="106"/>
       <x:c r="DW162" s="106"/>
+      <x:c r="DX162" s="109"/>
     </x:row>
     <x:row r="163" ht="25" customHeight="1">
       <x:c r="A163" s="10"/>
@@ -22215,6 +22560,7 @@
       <x:c r="DU163" s="106"/>
       <x:c r="DV163" s="106"/>
       <x:c r="DW163" s="106"/>
+      <x:c r="DX163" s="109"/>
     </x:row>
     <x:row r="164" ht="25" customHeight="1">
       <x:c r="A164" s="10"/>
@@ -22304,6 +22650,7 @@
       <x:c r="DU164" s="106"/>
       <x:c r="DV164" s="106"/>
       <x:c r="DW164" s="106"/>
+      <x:c r="DX164" s="109"/>
     </x:row>
     <x:row r="165" ht="25" customHeight="1">
       <x:c r="A165" s="10"/>
@@ -22393,6 +22740,7 @@
       <x:c r="DU165" s="106"/>
       <x:c r="DV165" s="106"/>
       <x:c r="DW165" s="106"/>
+      <x:c r="DX165" s="109"/>
     </x:row>
     <x:row r="166" ht="25" customHeight="1">
       <x:c r="A166" s="10"/>
@@ -22482,6 +22830,7 @@
       <x:c r="DU166" s="106"/>
       <x:c r="DV166" s="106"/>
       <x:c r="DW166" s="106"/>
+      <x:c r="DX166" s="109"/>
     </x:row>
     <x:row r="167" ht="25" customHeight="1">
       <x:c r="A167" s="10"/>
@@ -22571,6 +22920,7 @@
       <x:c r="DU167" s="106"/>
       <x:c r="DV167" s="106"/>
       <x:c r="DW167" s="106"/>
+      <x:c r="DX167" s="109"/>
     </x:row>
     <x:row r="168" ht="25" customHeight="1">
       <x:c r="A168" s="10"/>
@@ -22660,6 +23010,7 @@
       <x:c r="DU168" s="106"/>
       <x:c r="DV168" s="106"/>
       <x:c r="DW168" s="106"/>
+      <x:c r="DX168" s="109"/>
     </x:row>
     <x:row r="169" ht="25" customHeight="1">
       <x:c r="A169" s="10"/>
@@ -22749,6 +23100,7 @@
       <x:c r="DU169" s="106"/>
       <x:c r="DV169" s="106"/>
       <x:c r="DW169" s="106"/>
+      <x:c r="DX169" s="109"/>
     </x:row>
     <x:row r="170" ht="25" customHeight="1">
       <x:c r="A170" s="10"/>
@@ -22838,6 +23190,7 @@
       <x:c r="DU170" s="106"/>
       <x:c r="DV170" s="106"/>
       <x:c r="DW170" s="106"/>
+      <x:c r="DX170" s="109"/>
     </x:row>
     <x:row r="171" ht="25" customHeight="1">
       <x:c r="A171" s="10"/>
@@ -22927,6 +23280,7 @@
       <x:c r="DU171" s="106"/>
       <x:c r="DV171" s="106"/>
       <x:c r="DW171" s="106"/>
+      <x:c r="DX171" s="109"/>
     </x:row>
     <x:row r="172" ht="25" customHeight="1">
       <x:c r="A172" s="10"/>
@@ -23016,6 +23370,7 @@
       <x:c r="DU172" s="106"/>
       <x:c r="DV172" s="106"/>
       <x:c r="DW172" s="106"/>
+      <x:c r="DX172" s="109"/>
     </x:row>
     <x:row r="173" ht="25" customHeight="1">
       <x:c r="A173" s="10"/>
@@ -23105,6 +23460,7 @@
       <x:c r="DU173" s="106"/>
       <x:c r="DV173" s="106"/>
       <x:c r="DW173" s="106"/>
+      <x:c r="DX173" s="109"/>
     </x:row>
     <x:row r="174" ht="25" customHeight="1">
       <x:c r="A174" s="10"/>
@@ -23194,6 +23550,7 @@
       <x:c r="DU174" s="106"/>
       <x:c r="DV174" s="106"/>
       <x:c r="DW174" s="106"/>
+      <x:c r="DX174" s="109"/>
     </x:row>
     <x:row r="175" ht="25" customHeight="1">
       <x:c r="A175" s="10"/>
@@ -23283,6 +23640,7 @@
       <x:c r="DU175" s="106"/>
       <x:c r="DV175" s="106"/>
       <x:c r="DW175" s="106"/>
+      <x:c r="DX175" s="109"/>
     </x:row>
     <x:row r="176" ht="25" customHeight="1">
       <x:c r="A176" s="10"/>
@@ -23372,6 +23730,7 @@
       <x:c r="DU176" s="106"/>
       <x:c r="DV176" s="106"/>
       <x:c r="DW176" s="106"/>
+      <x:c r="DX176" s="109"/>
     </x:row>
     <x:row r="177" ht="25" customHeight="1">
       <x:c r="A177" s="10"/>
@@ -23461,6 +23820,7 @@
       <x:c r="DU177" s="106"/>
       <x:c r="DV177" s="106"/>
       <x:c r="DW177" s="106"/>
+      <x:c r="DX177" s="109"/>
     </x:row>
     <x:row r="178" ht="25" customHeight="1">
       <x:c r="A178" s="10"/>
@@ -23550,6 +23910,7 @@
       <x:c r="DU178" s="106"/>
       <x:c r="DV178" s="106"/>
       <x:c r="DW178" s="106"/>
+      <x:c r="DX178" s="109"/>
     </x:row>
     <x:row r="179" ht="25" customHeight="1">
       <x:c r="A179" s="10"/>
@@ -23639,6 +24000,7 @@
       <x:c r="DU179" s="106"/>
       <x:c r="DV179" s="106"/>
       <x:c r="DW179" s="106"/>
+      <x:c r="DX179" s="109"/>
     </x:row>
     <x:row r="180" ht="25" customHeight="1">
       <x:c r="A180" s="10"/>
@@ -23728,6 +24090,7 @@
       <x:c r="DU180" s="106"/>
       <x:c r="DV180" s="106"/>
       <x:c r="DW180" s="106"/>
+      <x:c r="DX180" s="109"/>
     </x:row>
     <x:row r="181" ht="25" customHeight="1">
       <x:c r="A181" s="10"/>
@@ -23817,6 +24180,7 @@
       <x:c r="DU181" s="106"/>
       <x:c r="DV181" s="106"/>
       <x:c r="DW181" s="106"/>
+      <x:c r="DX181" s="109"/>
     </x:row>
     <x:row r="182" ht="25" customHeight="1">
       <x:c r="A182" s="10"/>
@@ -23906,6 +24270,7 @@
       <x:c r="DU182" s="106"/>
       <x:c r="DV182" s="106"/>
       <x:c r="DW182" s="106"/>
+      <x:c r="DX182" s="109"/>
     </x:row>
     <x:row r="183" ht="25" customHeight="1">
       <x:c r="A183" s="10"/>
@@ -23995,6 +24360,7 @@
       <x:c r="DU183" s="106"/>
       <x:c r="DV183" s="106"/>
       <x:c r="DW183" s="106"/>
+      <x:c r="DX183" s="109"/>
     </x:row>
     <x:row r="184" ht="25" customHeight="1">
       <x:c r="A184" s="10"/>
@@ -24084,6 +24450,7 @@
       <x:c r="DU184" s="106"/>
       <x:c r="DV184" s="106"/>
       <x:c r="DW184" s="106"/>
+      <x:c r="DX184" s="109"/>
     </x:row>
     <x:row r="185" ht="25" customHeight="1">
       <x:c r="A185" s="10"/>
@@ -24173,6 +24540,7 @@
       <x:c r="DU185" s="106"/>
       <x:c r="DV185" s="106"/>
       <x:c r="DW185" s="106"/>
+      <x:c r="DX185" s="109"/>
     </x:row>
     <x:row r="186" ht="25" customHeight="1">
       <x:c r="A186" s="10"/>
@@ -24262,6 +24630,7 @@
       <x:c r="DU186" s="106"/>
       <x:c r="DV186" s="106"/>
       <x:c r="DW186" s="106"/>
+      <x:c r="DX186" s="109"/>
     </x:row>
     <x:row r="187" ht="25" customHeight="1">
       <x:c r="A187" s="10"/>
@@ -24351,6 +24720,7 @@
       <x:c r="DU187" s="106"/>
       <x:c r="DV187" s="106"/>
       <x:c r="DW187" s="106"/>
+      <x:c r="DX187" s="109"/>
     </x:row>
     <x:row r="188" ht="25" customHeight="1">
       <x:c r="A188" s="10"/>
@@ -24440,6 +24810,7 @@
       <x:c r="DU188" s="106"/>
       <x:c r="DV188" s="106"/>
       <x:c r="DW188" s="106"/>
+      <x:c r="DX188" s="109"/>
     </x:row>
     <x:row r="189" ht="25" customHeight="1">
       <x:c r="A189" s="10"/>
@@ -24529,6 +24900,7 @@
       <x:c r="DU189" s="106"/>
       <x:c r="DV189" s="106"/>
       <x:c r="DW189" s="106"/>
+      <x:c r="DX189" s="109"/>
     </x:row>
     <x:row r="190" ht="25" customHeight="1">
       <x:c r="A190" s="10"/>
@@ -24618,6 +24990,7 @@
       <x:c r="DU190" s="106"/>
       <x:c r="DV190" s="106"/>
       <x:c r="DW190" s="106"/>
+      <x:c r="DX190" s="109"/>
     </x:row>
     <x:row r="191" ht="25" customHeight="1">
       <x:c r="A191" s="10"/>
@@ -24707,6 +25080,7 @@
       <x:c r="DU191" s="106"/>
       <x:c r="DV191" s="106"/>
       <x:c r="DW191" s="106"/>
+      <x:c r="DX191" s="109"/>
     </x:row>
     <x:row r="192" ht="25" customHeight="1">
       <x:c r="A192" s="10"/>
@@ -24796,6 +25170,7 @@
       <x:c r="DU192" s="106"/>
       <x:c r="DV192" s="106"/>
       <x:c r="DW192" s="106"/>
+      <x:c r="DX192" s="109"/>
     </x:row>
     <x:row r="193" ht="25" customHeight="1">
       <x:c r="A193" s="10"/>
@@ -24885,6 +25260,7 @@
       <x:c r="DU193" s="106"/>
       <x:c r="DV193" s="106"/>
       <x:c r="DW193" s="106"/>
+      <x:c r="DX193" s="109"/>
     </x:row>
     <x:row r="194" ht="25" customHeight="1">
       <x:c r="A194" s="10"/>
@@ -24974,6 +25350,7 @@
       <x:c r="DU194" s="106"/>
       <x:c r="DV194" s="106"/>
       <x:c r="DW194" s="106"/>
+      <x:c r="DX194" s="109"/>
     </x:row>
     <x:row r="195" ht="25" customHeight="1">
       <x:c r="A195" s="10"/>
@@ -25063,6 +25440,7 @@
       <x:c r="DU195" s="106"/>
       <x:c r="DV195" s="106"/>
       <x:c r="DW195" s="106"/>
+      <x:c r="DX195" s="109"/>
     </x:row>
     <x:row r="196" ht="25" customHeight="1">
       <x:c r="A196" s="10"/>
@@ -25152,6 +25530,7 @@
       <x:c r="DU196" s="106"/>
       <x:c r="DV196" s="106"/>
       <x:c r="DW196" s="106"/>
+      <x:c r="DX196" s="109"/>
     </x:row>
     <x:row r="197" ht="25" customHeight="1">
       <x:c r="A197" s="10"/>
@@ -25241,6 +25620,7 @@
       <x:c r="DU197" s="106"/>
       <x:c r="DV197" s="106"/>
       <x:c r="DW197" s="106"/>
+      <x:c r="DX197" s="109"/>
     </x:row>
     <x:row r="198" ht="25" customHeight="1">
       <x:c r="A198" s="10"/>
@@ -25330,6 +25710,7 @@
       <x:c r="DU198" s="106"/>
       <x:c r="DV198" s="106"/>
       <x:c r="DW198" s="106"/>
+      <x:c r="DX198" s="109"/>
     </x:row>
     <x:row r="199" ht="25" customHeight="1">
       <x:c r="A199" s="10"/>
@@ -25419,6 +25800,7 @@
       <x:c r="DU199" s="106"/>
       <x:c r="DV199" s="106"/>
       <x:c r="DW199" s="106"/>
+      <x:c r="DX199" s="109"/>
     </x:row>
     <x:row r="200" ht="25" customHeight="1">
       <x:c r="A200" s="10"/>
@@ -25508,9 +25890,10 @@
       <x:c r="DU200" s="106"/>
       <x:c r="DV200" s="106"/>
       <x:c r="DW200" s="106"/>
+      <x:c r="DX200" s="109"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="48">
+  <x:dataValidations count="49">
     <x:dataValidation type="list" sqref="K2:K200">
       <x:formula1>"自身,敵一体,味方一体,自身中心,敵中心"</x:formula1>
     </x:dataValidation>
@@ -25657,10 +26040,13 @@
       <x:formula1>0.01</x:formula1>
       <x:formula2>1</x:formula2>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="DT2:DT200">
+      <x:formula1>"光の弾,衝撃波,魔方陣,斬撃,光の柱,煙と粒子,固有スプライト"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6846b5e35f994260"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R857149f39ec44096"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25776,7 +26162,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7276936c4c154f83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc36efa74d9a4e41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -29149,7 +29535,7 @@
         <x:v>画像設定</x:v>
       </x:c>
       <x:c r="B276" s="89" t="str">
-        <x:v>発射物_画像番号（右端DT列）</x:v>
+        <x:v>発射物_素材（DT）／固有スプライト（DX）（右端DT列）</x:v>
       </x:c>
       <x:c r="C276" s="89" t="str">
         <x:v>空欄ならスキルIDと同じ番号。別の正の整数も可</x:v>
@@ -29408,6 +29794,174 @@
       </x:c>
       <x:c r="D295" s="89" t="str">
         <x:v>既存範囲スキルの自動調整はコード反映後から有効</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="298" ht="48" customHeight="1">
+      <x:c r="A298" s="142" t="str">
+        <x:v>共通素材と固有スプライト</x:v>
+      </x:c>
+      <x:c r="B298" s="142" t="str">
+        <x:v>列</x:v>
+      </x:c>
+      <x:c r="C298" s="142" t="str">
+        <x:v>設定方法</x:v>
+      </x:c>
+      <x:c r="D298" s="142" t="str">
+        <x:v>例</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="299" ht="48" customHeight="1">
+      <x:c r="A299" s="89" t="str">
+        <x:v>共通素材</x:v>
+      </x:c>
+      <x:c r="B299" s="89" t="str">
+        <x:v>DT：発射物_素材</x:v>
+      </x:c>
+      <x:c r="C299" s="89" t="str">
+        <x:v>6種類または固有スプライトを選択</x:v>
+      </x:c>
+      <x:c r="D299" s="89" t="str">
+        <x:v>光の弾／衝撃波／魔方陣／斬撃／光の柱／煙と粒子</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="300" ht="48" customHeight="1">
+      <x:c r="A300" s="89" t="str">
+        <x:v>画像の配置</x:v>
+      </x:c>
+      <x:c r="B300" s="89" t="str">
+        <x:v>Assets/素材/Projectile</x:v>
+      </x:c>
+      <x:c r="C300" s="89" t="str">
+        <x:v>光の弾.png または 1.光の弾.png のように配置</x:v>
+      </x:c>
+      <x:c r="D300" s="89" t="str">
+        <x:v>番号だけの1.png～6.pngも対応。名前付き画像を優先</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="301" ht="48" customHeight="1">
+      <x:c r="A301" s="89" t="str">
+        <x:v>固有画像</x:v>
+      </x:c>
+      <x:c r="B301" s="89" t="str">
+        <x:v>DX：発射物_固有スプライト</x:v>
+      </x:c>
+      <x:c r="C301" s="89" t="str">
+        <x:v>DTで固有スプライトを選び、DXに画像名またはパス</x:v>
+      </x:c>
+      <x:c r="D301" s="89" t="str">
+        <x:v>Assets/素材/Projectile/固有/竜の炎.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="302" ht="48" customHeight="1">
+      <x:c r="A302" s="89" t="str">
+        <x:v>複数Sprite画像</x:v>
+      </x:c>
+      <x:c r="B302" s="89" t="str">
+        <x:v>DX：発射物_固有スプライト</x:v>
+      </x:c>
+      <x:c r="C302" s="89" t="str">
+        <x:v>アセットパスの後に #Sprite名 を付ける</x:v>
+      </x:c>
+      <x:c r="D302" s="89" t="str">
+        <x:v>Assets/素材/Projectile/固有/炎.png#炎_0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="303" ht="48" customHeight="1">
+      <x:c r="A303" s="89" t="str">
+        <x:v>名前の重複</x:v>
+      </x:c>
+      <x:c r="B303" s="89" t="str">
+        <x:v>DX：発射物_固有スプライト</x:v>
+      </x:c>
+      <x:c r="C303" s="89" t="str">
+        <x:v>同じ画像名がある場合はアセットパスで指定</x:v>
+      </x:c>
+      <x:c r="D303" s="89" t="str">
+        <x:v>指定が曖昧な場合は取り込み前にエラー</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="304" ht="48" customHeight="1">
+      <x:c r="A304" s="89" t="str">
+        <x:v>表示色</x:v>
+      </x:c>
+      <x:c r="B304" s="89" t="str">
+        <x:v>DF：発射物_色</x:v>
+      </x:c>
+      <x:c r="C304" s="89" t="str">
+        <x:v>#RRGGBB または #RRGGBBAA。白素材に乗算</x:v>
+      </x:c>
+      <x:c r="D304" s="89" t="str">
+        <x:v>火：#FF703FFF／水：#72DBFFFF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="305" ht="48" customHeight="1">
+      <x:c r="A305" s="89" t="str">
+        <x:v>透明度</x:v>
+      </x:c>
+      <x:c r="B305" s="89" t="str">
+        <x:v>DF：発射物_色</x:v>
+      </x:c>
+      <x:c r="C305" s="89" t="str">
+        <x:v>末尾AA。FF＝不透明、B3＝約70％、00＝透明</x:v>
+      </x:c>
+      <x:c r="D305" s="89" t="str">
+        <x:v>陣はB3～CC、弾はFFに再設定</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="306" ht="48" customHeight="1">
+      <x:c r="A306" s="89" t="str">
+        <x:v>元の色を保持</x:v>
+      </x:c>
+      <x:c r="B306" s="89" t="str">
+        <x:v>DF：発射物_色</x:v>
+      </x:c>
+      <x:c r="C306" s="89" t="str">
+        <x:v>色付き固有画像は白を指定</x:v>
+      </x:c>
+      <x:c r="D306" s="89" t="str">
+        <x:v>固有スプライト ＋ #FFFFFFFF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="307" ht="48" customHeight="1">
+      <x:c r="A307" s="89" t="str">
+        <x:v>表示サイズ</x:v>
+      </x:c>
+      <x:c r="B307" s="89" t="str">
+        <x:v>DE・DU列</x:v>
+      </x:c>
+      <x:c r="C307" s="89" t="str">
+        <x:v>弾は表示倍率、範囲技は範囲への自動調整を使用</x:v>
+      </x:c>
+      <x:c r="D307" s="89" t="str">
+        <x:v>素材を変えてもダメージ範囲は変わらない</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="308" ht="48" customHeight="1">
+      <x:c r="A308" s="89" t="str">
+        <x:v>旧Excel互換</x:v>
+      </x:c>
+      <x:c r="B308" s="89" t="str">
+        <x:v>旧：発射物_画像番号</x:v>
+      </x:c>
+      <x:c r="C308" s="89" t="str">
+        <x:v>新しい素材列が空なら旧画像番号、未指定ならスキルID</x:v>
+      </x:c>
+      <x:c r="D308" s="89" t="str">
+        <x:v>旧列は新テンプレートでは素材選択列へ変更</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="309" ht="48" customHeight="1">
+      <x:c r="A309" s="89" t="str">
+        <x:v>反映方法</x:v>
+      </x:c>
+      <x:c r="B309" s="89" t="str">
+        <x:v>スキル取り込み</x:v>
+      </x:c>
+      <x:c r="C309" s="89" t="str">
+        <x:v>更新Excelを取り込むと既存Prefabの画像・色を更新</x:v>
+      </x:c>
+      <x:c r="D309" s="89" t="str">
+        <x:v>PrefabのID・参照は維持</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>